<commit_message>
Add excel_to_cdd.py to write Excel edits back into a CDD
The Excel export now carries ref columns that link each row to its CDD
element. excel_to_cdd.py uses the original CDD as the template, rewrites
only the changed values in place (keeping ids, quotes and line endings),
validates every edit, reads the result back to check it, and writes no
CDD when there are errors.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZDtTEV2ArMJ1VjWmCEQnF
</commit_message>
<xml_diff>
--- a/Cdd Parsing/RADAR_G7_CHERY03_APP_and_BOOT.xlsx
+++ b/Cdd Parsing/RADAR_G7_CHERY03_APP_and_BOOT.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RID" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Service'!$A$1:$K$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DID'!$A$1:$Y$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DTC'!$A$1:$AB$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RID'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Service'!$A$1:$L$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DID'!$A$1:$AA$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DTC'!$A$1:$AC$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RID'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,7 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +509,11 @@
           <t>Security</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CDD Ref</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -565,6 +571,11 @@
           <t>Locked, Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>_2998@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -622,6 +633,11 @@
           <t>Locked, Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>_3000@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -679,6 +695,11 @@
           <t>Locked, Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>_3002@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -736,6 +757,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>_3004@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -793,6 +819,11 @@
           <t>Locked, Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>_3007@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -850,6 +881,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>_3009@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -907,6 +943,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>_3010@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -964,6 +1005,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>_3011@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1021,6 +1067,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>_3012@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1078,6 +1129,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>_3013@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1135,6 +1191,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>_3014@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1192,6 +1253,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>_3017@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1249,6 +1315,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>_3019@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1306,6 +1377,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>_3021@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1363,6 +1439,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>_3022@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1420,6 +1501,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>_3029@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1477,6 +1563,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>_3030@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1534,6 +1625,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>_3031@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1591,6 +1687,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>_3033@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1648,6 +1749,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>_3034@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1705,6 +1811,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>_3035@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1762,6 +1873,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>_3037@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1819,6 +1935,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>_3038@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1876,6 +1997,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>_3039@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1933,6 +2059,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>_3041@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1990,6 +2121,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>_3042@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2047,6 +2183,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>_3043@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2104,6 +2245,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>_3045@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2161,6 +2307,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>_3046@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2218,6 +2369,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>_3047@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2275,6 +2431,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>_3049@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2332,6 +2493,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>_3050@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2389,6 +2555,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>_3051@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2446,6 +2617,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>_3004@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2503,6 +2679,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>_3058@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2560,6 +2741,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>_3060@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2617,6 +2803,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>_3063@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2674,6 +2865,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>_3021@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2731,6 +2927,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>_3022@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2788,6 +2989,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>_3065@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2845,6 +3051,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>_3066@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2902,6 +3113,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>_3067@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2959,6 +3175,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>_3068@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3016,6 +3237,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>_3069@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3073,6 +3299,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>_3070@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3130,6 +3361,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>_3071@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3187,6 +3423,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>_3072@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3244,6 +3485,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>_3073@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3301,6 +3547,11 @@
           <t>Unlocked_0x11</t>
         </is>
       </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>_3074@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3358,6 +3609,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>_3075@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3415,6 +3671,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>_3076@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3472,6 +3733,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>_3077@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3529,6 +3795,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>_3078@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3586,6 +3857,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>_3079@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3643,6 +3919,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>_3080@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3700,6 +3981,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>_3081@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3757,6 +4043,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>_3082@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3814,6 +4105,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>_3083@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3871,6 +4167,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>_3084@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3928,6 +4229,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>_3085@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3985,6 +4291,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>_3086@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4042,6 +4353,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>_3087@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4099,6 +4415,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>_3088@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4156,6 +4477,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>_3089@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4213,6 +4539,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>_3090@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4270,6 +4601,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>_3091@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4327,6 +4663,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>_3092@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4384,6 +4725,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>_3094@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4441,6 +4787,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>_3095@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4498,6 +4849,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>_3096@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4555,6 +4911,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>_3097@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4612,6 +4973,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>_3098@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4669,6 +5035,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>_3099@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4726,6 +5097,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>_3100@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4783,6 +5159,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>_3101@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4840,6 +5221,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>_3102@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4897,6 +5283,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>_3105@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4954,6 +5345,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>_3106@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5011,6 +5407,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>_3107@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5068,6 +5469,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>_3108@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5125,6 +5531,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>_3109@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5182,6 +5593,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>_3110@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5239,6 +5655,11 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>_3113@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5296,6 +5717,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>_3115@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5353,6 +5779,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>_3116@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5410,6 +5841,11 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>_3117@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5467,6 +5903,11 @@
           <t>Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>_3119@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5524,6 +5965,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>_3120@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5581,6 +6027,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>_3122@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5638,6 +6089,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>_3123@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5695,6 +6151,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>_3124@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5752,6 +6213,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>_3125@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5809,6 +6275,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>_3126@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5866,6 +6337,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>_3004@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5923,6 +6399,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>_3164@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5980,6 +6461,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>_3166@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -6037,6 +6523,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>_3009@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -6094,6 +6585,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>_3010@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -6151,6 +6647,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>_3011@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6208,6 +6709,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>_3012@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6265,6 +6771,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>_3013@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6322,6 +6833,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>_3014@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -6379,6 +6895,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>_3169@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6436,6 +6957,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>_3021@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6493,6 +7019,11 @@
           <t>Locked, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>_3022@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6550,6 +7081,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>_3172@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6607,6 +7143,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>_3173@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -6664,6 +7205,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>_3174@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6721,6 +7267,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>_3175@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6778,6 +7329,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>_3176@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6835,6 +7391,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>_3177@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6892,6 +7453,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>_3179@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6949,6 +7515,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>_3181@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -7006,6 +7577,11 @@
           <t>All</t>
         </is>
       </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>_3183@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -7063,6 +7639,11 @@
           <t>Locked, Unlocked_0x11</t>
         </is>
       </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>_3187@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -7120,6 +7701,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>_3189@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -7177,6 +7763,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>_3191@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -7234,6 +7825,11 @@
           <t>Unlocked_0x11</t>
         </is>
       </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>_3193@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7291,6 +7887,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>_3195@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7348,6 +7949,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>_3197@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7405,6 +8011,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>_3199@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7462,6 +8073,11 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>_3201@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7519,6 +8135,11 @@
           <t>Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>_3203@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -7576,6 +8197,11 @@
           <t>Unlocked_0x11, Unlocked_0x1</t>
         </is>
       </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>_3204@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -7633,6 +8259,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>_3206@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7690,6 +8321,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>_3207@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -7747,6 +8383,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>_3208@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -7804,6 +8445,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>_3209@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -7861,6 +8507,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>_3210@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7918,6 +8569,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>_3211@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7975,6 +8631,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>_3212@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -8032,6 +8693,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>_3213@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -8089,6 +8755,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>_3214@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8146,6 +8817,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>_3215@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -8203,6 +8879,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>_3216@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -8260,6 +8941,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>_3217@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -8317,6 +9003,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>_3218@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -8374,6 +9065,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>_3219@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8431,9 +9127,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>_3220@_3159</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K140"/>
+  <autoFilter ref="A1:L140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8444,7 +9145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y100"/>
+  <dimension ref="A1:AA100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8472,6 +9173,8 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="27" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8598,6 +9301,16 @@
       <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Write Security</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>DID Ref</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Element Ref</t>
         </is>
       </c>
     </row>
@@ -8703,6 +9416,16 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>_1142</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>_1142:0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -8798,6 +9521,16 @@
       </c>
       <c r="X3" s="2" t="inlineStr"/>
       <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>_1143</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>_1143:0</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -8898,6 +9631,16 @@
       </c>
       <c r="X4" s="2" t="inlineStr"/>
       <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>_1144</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>_1144:0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9001,6 +9744,16 @@
       </c>
       <c r="X5" s="2" t="inlineStr"/>
       <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>_1145</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>_1145:0</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9103,6 +9856,16 @@
       </c>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>_1146</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>_1146:0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -9198,6 +9961,16 @@
       </c>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>_1146</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>_1146:1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9298,6 +10071,16 @@
       </c>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>_1147</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>_1147:0</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -9412,6 +10195,16 @@
       </c>
       <c r="X9" s="2" t="inlineStr"/>
       <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>_1148</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>_1148:0</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9515,6 +10308,16 @@
       </c>
       <c r="X10" s="2" t="inlineStr"/>
       <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>_1149:0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9618,6 +10421,16 @@
       </c>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>_1149:1</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9719,6 +10532,16 @@
       </c>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>_1149:2</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9822,6 +10645,16 @@
       </c>
       <c r="X13" s="2" t="inlineStr"/>
       <c r="Y13" s="2" t="inlineStr"/>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>_1149:3</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9925,6 +10758,16 @@
       </c>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>_1149:4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -10028,6 +10871,16 @@
       </c>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>_1149:5</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -10127,6 +10980,16 @@
       </c>
       <c r="X16" s="2" t="inlineStr"/>
       <c r="Y16" s="2" t="inlineStr"/>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>_1149:6</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -10226,6 +11089,16 @@
       </c>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>_1149:7</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -10325,6 +11198,16 @@
       </c>
       <c r="X18" s="2" t="inlineStr"/>
       <c r="Y18" s="2" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA18" s="2" t="inlineStr">
+        <is>
+          <t>_1149:8</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -10424,6 +11307,16 @@
       </c>
       <c r="X19" s="2" t="inlineStr"/>
       <c r="Y19" s="2" t="inlineStr"/>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>_1149:9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -10527,6 +11420,16 @@
       </c>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="inlineStr"/>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>_1149:10</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -10630,6 +11533,16 @@
       </c>
       <c r="X21" s="2" t="inlineStr"/>
       <c r="Y21" s="2" t="inlineStr"/>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>_1149:11</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -10733,6 +11646,16 @@
       </c>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="2" t="inlineStr"/>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>_1149:12</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -10828,6 +11751,16 @@
       </c>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>_1149</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>_1149:13</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -10927,6 +11860,16 @@
       </c>
       <c r="X24" s="2" t="inlineStr"/>
       <c r="Y24" s="2" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>_1150:0</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -11026,6 +11969,16 @@
       </c>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>_1150:1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -11125,6 +12078,16 @@
       </c>
       <c r="X26" s="2" t="inlineStr"/>
       <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>_1150:2</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -11228,6 +12191,16 @@
       </c>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>_1150:3</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -11331,6 +12304,16 @@
       </c>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>_1150:4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11434,6 +12417,16 @@
       </c>
       <c r="X29" s="2" t="inlineStr"/>
       <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>_1150</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>_1150:5</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11537,6 +12530,16 @@
       </c>
       <c r="X30" s="2" t="inlineStr"/>
       <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>_1151</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>_1151:0</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11640,6 +12643,16 @@
       </c>
       <c r="X31" s="2" t="inlineStr"/>
       <c r="Y31" s="2" t="inlineStr"/>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>_1152</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>_1152:0</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11743,6 +12756,16 @@
       </c>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="inlineStr"/>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>_1153</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>_1153:0</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11838,6 +12861,16 @@
       </c>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="2" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>_1154</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>_1154:0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11933,6 +12966,16 @@
       </c>
       <c r="X34" s="2" t="inlineStr"/>
       <c r="Y34" s="2" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>_1155</t>
+        </is>
+      </c>
+      <c r="AA34" s="2" t="inlineStr">
+        <is>
+          <t>_1155:0</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12028,6 +13071,16 @@
           <t>All</t>
         </is>
       </c>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>_1156</t>
+        </is>
+      </c>
+      <c r="AA35" s="2" t="inlineStr">
+        <is>
+          <t>_1156:0</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12123,6 +13176,16 @@
       </c>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="inlineStr"/>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>_1157</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>_1157:0</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12218,6 +13281,16 @@
       </c>
       <c r="X37" s="2" t="inlineStr"/>
       <c r="Y37" s="2" t="inlineStr"/>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>_1158</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>_1158:0</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12313,6 +13386,16 @@
       </c>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
+          <t>_1159</t>
+        </is>
+      </c>
+      <c r="AA38" s="2" t="inlineStr">
+        <is>
+          <t>_1159:0</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12408,6 +13491,16 @@
       </c>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="2" t="inlineStr"/>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>_1160:0</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12503,6 +13596,16 @@
       </c>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="inlineStr"/>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>_1160:1</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12598,6 +13701,16 @@
       </c>
       <c r="X41" s="2" t="inlineStr"/>
       <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>_1160:2</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12693,6 +13806,16 @@
       </c>
       <c r="X42" s="2" t="inlineStr"/>
       <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>_1160:3</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12788,6 +13911,16 @@
       </c>
       <c r="X43" s="2" t="inlineStr"/>
       <c r="Y43" s="2" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA43" s="2" t="inlineStr">
+        <is>
+          <t>_1160:4</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12883,6 +14016,16 @@
       </c>
       <c r="X44" s="2" t="inlineStr"/>
       <c r="Y44" s="2" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA44" s="2" t="inlineStr">
+        <is>
+          <t>_1160:5</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12978,6 +14121,16 @@
       </c>
       <c r="X45" s="2" t="inlineStr"/>
       <c r="Y45" s="2" t="inlineStr"/>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>_1160:6</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13073,6 +14226,16 @@
       </c>
       <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr"/>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>_1160:7</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13168,6 +14331,16 @@
       </c>
       <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA47" s="2" t="inlineStr">
+        <is>
+          <t>_1160:8</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13263,6 +14436,16 @@
       </c>
       <c r="X48" s="2" t="inlineStr"/>
       <c r="Y48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>_1160:9</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13358,6 +14541,16 @@
       </c>
       <c r="X49" s="2" t="inlineStr"/>
       <c r="Y49" s="2" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA49" s="2" t="inlineStr">
+        <is>
+          <t>_1160:10</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13453,6 +14646,16 @@
       </c>
       <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA50" s="2" t="inlineStr">
+        <is>
+          <t>_1160:11</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13548,6 +14751,16 @@
       </c>
       <c r="X51" s="2" t="inlineStr"/>
       <c r="Y51" s="2" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA51" s="2" t="inlineStr">
+        <is>
+          <t>_1160:12</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13643,6 +14856,16 @@
       </c>
       <c r="X52" s="2" t="inlineStr"/>
       <c r="Y52" s="2" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA52" s="2" t="inlineStr">
+        <is>
+          <t>_1160:13</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13738,6 +14961,16 @@
       </c>
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr"/>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>_1160:14</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13833,6 +15066,16 @@
       </c>
       <c r="X54" s="2" t="inlineStr"/>
       <c r="Y54" s="2" t="inlineStr"/>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>_1160:15</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13928,6 +15171,16 @@
       </c>
       <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA55" s="2" t="inlineStr">
+        <is>
+          <t>_1160:16</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14023,6 +15276,16 @@
       </c>
       <c r="X56" s="2" t="inlineStr"/>
       <c r="Y56" s="2" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>_1160:17</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14118,6 +15381,16 @@
       </c>
       <c r="X57" s="2" t="inlineStr"/>
       <c r="Y57" s="2" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>_1160:18</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14213,6 +15486,16 @@
       </c>
       <c r="X58" s="2" t="inlineStr"/>
       <c r="Y58" s="2" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>_1160:19</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14308,6 +15591,16 @@
       </c>
       <c r="X59" s="2" t="inlineStr"/>
       <c r="Y59" s="2" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA59" s="2" t="inlineStr">
+        <is>
+          <t>_1160:20</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14403,6 +15696,16 @@
       </c>
       <c r="X60" s="2" t="inlineStr"/>
       <c r="Y60" s="2" t="inlineStr"/>
+      <c r="Z60" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA60" s="2" t="inlineStr">
+        <is>
+          <t>_1160:21</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14498,6 +15801,16 @@
       </c>
       <c r="X61" s="2" t="inlineStr"/>
       <c r="Y61" s="2" t="inlineStr"/>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>_1160</t>
+        </is>
+      </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>_1160:22</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14598,6 +15911,16 @@
       </c>
       <c r="X62" s="2" t="inlineStr"/>
       <c r="Y62" s="2" t="inlineStr"/>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>_1161</t>
+        </is>
+      </c>
+      <c r="AA62" s="2" t="inlineStr">
+        <is>
+          <t>_1161:0</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -14697,6 +16020,16 @@
       </c>
       <c r="X63" s="2" t="inlineStr"/>
       <c r="Y63" s="2" t="inlineStr"/>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>_1162</t>
+        </is>
+      </c>
+      <c r="AA63" s="2" t="inlineStr">
+        <is>
+          <t>_1162:0</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -14796,6 +16129,16 @@
       </c>
       <c r="X64" s="2" t="inlineStr"/>
       <c r="Y64" s="2" t="inlineStr"/>
+      <c r="Z64" s="2" t="inlineStr">
+        <is>
+          <t>_1163</t>
+        </is>
+      </c>
+      <c r="AA64" s="2" t="inlineStr">
+        <is>
+          <t>_1163:0</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -14891,6 +16234,16 @@
       </c>
       <c r="X65" s="2" t="inlineStr"/>
       <c r="Y65" s="2" t="inlineStr"/>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
+          <t>_1164</t>
+        </is>
+      </c>
+      <c r="AA65" s="2" t="inlineStr">
+        <is>
+          <t>_1164:0</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -14986,6 +16339,16 @@
       </c>
       <c r="X66" s="2" t="inlineStr"/>
       <c r="Y66" s="2" t="inlineStr"/>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>_1164</t>
+        </is>
+      </c>
+      <c r="AA66" s="2" t="inlineStr">
+        <is>
+          <t>_1164:1</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -15081,6 +16444,16 @@
       </c>
       <c r="X67" s="2" t="inlineStr"/>
       <c r="Y67" s="2" t="inlineStr"/>
+      <c r="Z67" s="2" t="inlineStr">
+        <is>
+          <t>_1165</t>
+        </is>
+      </c>
+      <c r="AA67" s="2" t="inlineStr">
+        <is>
+          <t>_1165:0</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -15176,6 +16549,16 @@
       </c>
       <c r="X68" s="2" t="inlineStr"/>
       <c r="Y68" s="2" t="inlineStr"/>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>_1165</t>
+        </is>
+      </c>
+      <c r="AA68" s="2" t="inlineStr">
+        <is>
+          <t>_1165:1</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -15271,6 +16654,16 @@
       </c>
       <c r="X69" s="2" t="inlineStr"/>
       <c r="Y69" s="2" t="inlineStr"/>
+      <c r="Z69" s="2" t="inlineStr">
+        <is>
+          <t>_1165</t>
+        </is>
+      </c>
+      <c r="AA69" s="2" t="inlineStr">
+        <is>
+          <t>_1165:2</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -15366,6 +16759,16 @@
       </c>
       <c r="X70" s="2" t="inlineStr"/>
       <c r="Y70" s="2" t="inlineStr"/>
+      <c r="Z70" s="2" t="inlineStr">
+        <is>
+          <t>_1165</t>
+        </is>
+      </c>
+      <c r="AA70" s="2" t="inlineStr">
+        <is>
+          <t>_1165:3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -15467,6 +16870,16 @@
       </c>
       <c r="X71" s="2" t="inlineStr"/>
       <c r="Y71" s="2" t="inlineStr"/>
+      <c r="Z71" s="2" t="inlineStr">
+        <is>
+          <t>_1166</t>
+        </is>
+      </c>
+      <c r="AA71" s="2" t="inlineStr">
+        <is>
+          <t>_1166:0</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -15562,6 +16975,16 @@
       </c>
       <c r="X72" s="2" t="inlineStr"/>
       <c r="Y72" s="2" t="inlineStr"/>
+      <c r="Z72" s="2" t="inlineStr">
+        <is>
+          <t>_1167</t>
+        </is>
+      </c>
+      <c r="AA72" s="2" t="inlineStr">
+        <is>
+          <t>_1167:0</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -15657,6 +17080,16 @@
       </c>
       <c r="X73" s="2" t="inlineStr"/>
       <c r="Y73" s="2" t="inlineStr"/>
+      <c r="Z73" s="2" t="inlineStr">
+        <is>
+          <t>_1167</t>
+        </is>
+      </c>
+      <c r="AA73" s="2" t="inlineStr">
+        <is>
+          <t>_1167:1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -15752,6 +17185,16 @@
       </c>
       <c r="X74" s="2" t="inlineStr"/>
       <c r="Y74" s="2" t="inlineStr"/>
+      <c r="Z74" s="2" t="inlineStr">
+        <is>
+          <t>_1167</t>
+        </is>
+      </c>
+      <c r="AA74" s="2" t="inlineStr">
+        <is>
+          <t>_1167:2</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -15847,6 +17290,16 @@
       </c>
       <c r="X75" s="2" t="inlineStr"/>
       <c r="Y75" s="2" t="inlineStr"/>
+      <c r="Z75" s="2" t="inlineStr">
+        <is>
+          <t>_1167</t>
+        </is>
+      </c>
+      <c r="AA75" s="2" t="inlineStr">
+        <is>
+          <t>_1167:3</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -15942,6 +17395,16 @@
       </c>
       <c r="X76" s="2" t="inlineStr"/>
       <c r="Y76" s="2" t="inlineStr"/>
+      <c r="Z76" s="2" t="inlineStr">
+        <is>
+          <t>_1167</t>
+        </is>
+      </c>
+      <c r="AA76" s="2" t="inlineStr">
+        <is>
+          <t>_1167:4</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -16037,6 +17500,16 @@
       </c>
       <c r="X77" s="2" t="inlineStr"/>
       <c r="Y77" s="2" t="inlineStr"/>
+      <c r="Z77" s="2" t="inlineStr">
+        <is>
+          <t>_1168</t>
+        </is>
+      </c>
+      <c r="AA77" s="2" t="inlineStr">
+        <is>
+          <t>_1168:0</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -16132,6 +17605,16 @@
       </c>
       <c r="X78" s="2" t="inlineStr"/>
       <c r="Y78" s="2" t="inlineStr"/>
+      <c r="Z78" s="2" t="inlineStr">
+        <is>
+          <t>_1168</t>
+        </is>
+      </c>
+      <c r="AA78" s="2" t="inlineStr">
+        <is>
+          <t>_1168:1</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -16227,6 +17710,16 @@
       </c>
       <c r="X79" s="2" t="inlineStr"/>
       <c r="Y79" s="2" t="inlineStr"/>
+      <c r="Z79" s="2" t="inlineStr">
+        <is>
+          <t>_1168</t>
+        </is>
+      </c>
+      <c r="AA79" s="2" t="inlineStr">
+        <is>
+          <t>_1168:2</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -16322,6 +17815,16 @@
       </c>
       <c r="X80" s="2" t="inlineStr"/>
       <c r="Y80" s="2" t="inlineStr"/>
+      <c r="Z80" s="2" t="inlineStr">
+        <is>
+          <t>_1168</t>
+        </is>
+      </c>
+      <c r="AA80" s="2" t="inlineStr">
+        <is>
+          <t>_1168:3</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -16417,6 +17920,16 @@
       </c>
       <c r="X81" s="2" t="inlineStr"/>
       <c r="Y81" s="2" t="inlineStr"/>
+      <c r="Z81" s="2" t="inlineStr">
+        <is>
+          <t>_1168</t>
+        </is>
+      </c>
+      <c r="AA81" s="2" t="inlineStr">
+        <is>
+          <t>_1168:4</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -16512,6 +18025,16 @@
       </c>
       <c r="X82" s="2" t="inlineStr"/>
       <c r="Y82" s="2" t="inlineStr"/>
+      <c r="Z82" s="2" t="inlineStr">
+        <is>
+          <t>_1169</t>
+        </is>
+      </c>
+      <c r="AA82" s="2" t="inlineStr">
+        <is>
+          <t>_1169:0</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -16607,6 +18130,16 @@
       </c>
       <c r="X83" s="2" t="inlineStr"/>
       <c r="Y83" s="2" t="inlineStr"/>
+      <c r="Z83" s="2" t="inlineStr">
+        <is>
+          <t>_1170</t>
+        </is>
+      </c>
+      <c r="AA83" s="2" t="inlineStr">
+        <is>
+          <t>_1170:0</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -16714,6 +18247,16 @@
           <t>Unlocked_0x11</t>
         </is>
       </c>
+      <c r="Z84" s="2" t="inlineStr">
+        <is>
+          <t>_1171</t>
+        </is>
+      </c>
+      <c r="AA84" s="2" t="inlineStr">
+        <is>
+          <t>_1171:0</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -16821,6 +18364,16 @@
           <t>Unlocked_0x11</t>
         </is>
       </c>
+      <c r="Z85" s="2" t="inlineStr">
+        <is>
+          <t>_1171</t>
+        </is>
+      </c>
+      <c r="AA85" s="2" t="inlineStr">
+        <is>
+          <t>_1171:1</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -16926,6 +18479,16 @@
       <c r="Y86" s="2" t="inlineStr">
         <is>
           <t>Unlocked_0x11</t>
+        </is>
+      </c>
+      <c r="Z86" s="2" t="inlineStr">
+        <is>
+          <t>_1171</t>
+        </is>
+      </c>
+      <c r="AA86" s="2" t="inlineStr">
+        <is>
+          <t>_1171:2</t>
         </is>
       </c>
     </row>
@@ -17031,6 +18594,16 @@
           <t>Unlocked_0x11</t>
         </is>
       </c>
+      <c r="Z87" s="2" t="inlineStr">
+        <is>
+          <t>_1171</t>
+        </is>
+      </c>
+      <c r="AA87" s="2" t="inlineStr">
+        <is>
+          <t>_1171:3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -17126,6 +18699,16 @@
       </c>
       <c r="X88" s="2" t="inlineStr"/>
       <c r="Y88" s="2" t="inlineStr"/>
+      <c r="Z88" s="2" t="inlineStr">
+        <is>
+          <t>_1172</t>
+        </is>
+      </c>
+      <c r="AA88" s="2" t="inlineStr">
+        <is>
+          <t>_1172:0</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -17221,6 +18804,16 @@
       </c>
       <c r="X89" s="2" t="inlineStr"/>
       <c r="Y89" s="2" t="inlineStr"/>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
+          <t>_1173</t>
+        </is>
+      </c>
+      <c r="AA89" s="2" t="inlineStr">
+        <is>
+          <t>_1173:0</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -17316,6 +18909,16 @@
       </c>
       <c r="X90" s="2" t="inlineStr"/>
       <c r="Y90" s="2" t="inlineStr"/>
+      <c r="Z90" s="2" t="inlineStr">
+        <is>
+          <t>_1174</t>
+        </is>
+      </c>
+      <c r="AA90" s="2" t="inlineStr">
+        <is>
+          <t>_1174:0</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -17411,6 +19014,16 @@
       </c>
       <c r="X91" s="2" t="inlineStr"/>
       <c r="Y91" s="2" t="inlineStr"/>
+      <c r="Z91" s="2" t="inlineStr">
+        <is>
+          <t>_1175</t>
+        </is>
+      </c>
+      <c r="AA91" s="2" t="inlineStr">
+        <is>
+          <t>_1175:0</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -17506,6 +19119,16 @@
       </c>
       <c r="X92" s="2" t="inlineStr"/>
       <c r="Y92" s="2" t="inlineStr"/>
+      <c r="Z92" s="2" t="inlineStr">
+        <is>
+          <t>_1176</t>
+        </is>
+      </c>
+      <c r="AA92" s="2" t="inlineStr">
+        <is>
+          <t>_1176:0</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -17601,6 +19224,16 @@
       </c>
       <c r="X93" s="2" t="inlineStr"/>
       <c r="Y93" s="2" t="inlineStr"/>
+      <c r="Z93" s="2" t="inlineStr">
+        <is>
+          <t>_1177</t>
+        </is>
+      </c>
+      <c r="AA93" s="2" t="inlineStr">
+        <is>
+          <t>_1177:0</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -17696,6 +19329,16 @@
       </c>
       <c r="X94" s="2" t="inlineStr"/>
       <c r="Y94" s="2" t="inlineStr"/>
+      <c r="Z94" s="2" t="inlineStr">
+        <is>
+          <t>_1178</t>
+        </is>
+      </c>
+      <c r="AA94" s="2" t="inlineStr">
+        <is>
+          <t>_1178:0</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -17791,6 +19434,16 @@
       </c>
       <c r="X95" s="2" t="inlineStr"/>
       <c r="Y95" s="2" t="inlineStr"/>
+      <c r="Z95" s="2" t="inlineStr">
+        <is>
+          <t>_1179</t>
+        </is>
+      </c>
+      <c r="AA95" s="2" t="inlineStr">
+        <is>
+          <t>_1179:0</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -17894,6 +19547,16 @@
           <t>Unlocked_0x1</t>
         </is>
       </c>
+      <c r="Z96" s="2" t="inlineStr">
+        <is>
+          <t>_1180</t>
+        </is>
+      </c>
+      <c r="AA96" s="2" t="inlineStr">
+        <is>
+          <t>_1180:0</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -17989,6 +19652,16 @@
       </c>
       <c r="X97" s="2" t="inlineStr"/>
       <c r="Y97" s="2" t="inlineStr"/>
+      <c r="Z97" s="2" t="inlineStr">
+        <is>
+          <t>_1181</t>
+        </is>
+      </c>
+      <c r="AA97" s="2" t="inlineStr">
+        <is>
+          <t>_1181:0</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -18084,6 +19757,16 @@
       </c>
       <c r="X98" s="2" t="inlineStr"/>
       <c r="Y98" s="2" t="inlineStr"/>
+      <c r="Z98" s="2" t="inlineStr">
+        <is>
+          <t>_1182</t>
+        </is>
+      </c>
+      <c r="AA98" s="2" t="inlineStr">
+        <is>
+          <t>_1182:0</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -18179,6 +19862,16 @@
       </c>
       <c r="X99" s="2" t="inlineStr"/>
       <c r="Y99" s="2" t="inlineStr"/>
+      <c r="Z99" s="2" t="inlineStr">
+        <is>
+          <t>_1183</t>
+        </is>
+      </c>
+      <c r="AA99" s="2" t="inlineStr">
+        <is>
+          <t>_1183:0</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -18274,9 +19967,19 @@
       </c>
       <c r="X100" s="2" t="inlineStr"/>
       <c r="Y100" s="2" t="inlineStr"/>
+      <c r="Z100" s="2" t="inlineStr">
+        <is>
+          <t>_1184</t>
+        </is>
+      </c>
+      <c r="AA100" s="2" t="inlineStr">
+        <is>
+          <t>_1184:0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y100"/>
+  <autoFilter ref="A1:AA100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18287,7 +19990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB34"/>
+  <dimension ref="A1:AC34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -18318,6 +20021,7 @@
     <col width="48" customWidth="1" min="26" max="26"/>
     <col width="40" customWidth="1" min="27" max="27"/>
     <col width="41" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18459,6 +20163,11 @@
       <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>DS_DTCExistingExtendedDataRecordNumbers</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>CDD Ref</t>
         </is>
       </c>
     </row>
@@ -18620,6 +20329,11 @@
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>_2986</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -18752,6 +20466,11 @@
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>_2987</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -18892,6 +20611,11 @@
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>_2988</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -19030,6 +20754,11 @@
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>_2989</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -19166,6 +20895,11 @@
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>_2990</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -19298,6 +21032,11 @@
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>_2991</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -19447,6 +21186,11 @@
         </is>
       </c>
       <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>_2992</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -19577,6 +21321,11 @@
         </is>
       </c>
       <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>_3128</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -19703,6 +21452,11 @@
         </is>
       </c>
       <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>_3129</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -19837,6 +21591,11 @@
         </is>
       </c>
       <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>_3130</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -19961,6 +21720,11 @@
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>_3131</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -20113,6 +21877,11 @@
           <t>tbd</t>
         </is>
       </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>_3132</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -20237,6 +22006,11 @@
         </is>
       </c>
       <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>_3133</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -20367,6 +22141,11 @@
         </is>
       </c>
       <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>_3134</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -20499,6 +22278,11 @@
         </is>
       </c>
       <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>_3135</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -20636,6 +22420,11 @@
         </is>
       </c>
       <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>_3136</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -20773,6 +22562,11 @@
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr"/>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>_3137</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -20909,6 +22703,11 @@
         </is>
       </c>
       <c r="AB19" s="2" t="inlineStr"/>
+      <c r="AC19" s="2" t="inlineStr">
+        <is>
+          <t>_3138</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -21046,6 +22845,11 @@
         </is>
       </c>
       <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AC20" s="2" t="inlineStr">
+        <is>
+          <t>_3139</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -21182,6 +22986,11 @@
         </is>
       </c>
       <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AC21" s="2" t="inlineStr">
+        <is>
+          <t>_3140</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -21318,6 +23127,11 @@
         </is>
       </c>
       <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>_3141</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -21485,6 +23299,11 @@
         </is>
       </c>
       <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>_3142</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -21625,6 +23444,11 @@
         </is>
       </c>
       <c r="AB24" s="2" t="inlineStr"/>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>_3143</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -21771,6 +23595,11 @@
         </is>
       </c>
       <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>_3144</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -21915,6 +23744,11 @@
         </is>
       </c>
       <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>_3145</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -22045,6 +23879,11 @@
         </is>
       </c>
       <c r="AB27" s="2" t="inlineStr"/>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>_3146</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -22196,6 +24035,11 @@
           <t>tbd</t>
         </is>
       </c>
+      <c r="AC28" s="2" t="inlineStr">
+        <is>
+          <t>_3147</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -22347,6 +24191,11 @@
           <t>tbd</t>
         </is>
       </c>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>_3148</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -22484,6 +24333,11 @@
         </is>
       </c>
       <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AC30" s="2" t="inlineStr">
+        <is>
+          <t>_3149</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -22606,6 +24460,11 @@
         </is>
       </c>
       <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AC31" s="2" t="inlineStr">
+        <is>
+          <t>_3150</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -22746,6 +24605,11 @@
         </is>
       </c>
       <c r="AB32" s="2" t="inlineStr"/>
+      <c r="AC32" s="2" t="inlineStr">
+        <is>
+          <t>_3151</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -22904,6 +24768,11 @@
         </is>
       </c>
       <c r="AB33" s="2" t="inlineStr"/>
+      <c r="AC33" s="2" t="inlineStr">
+        <is>
+          <t>_3152</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -23060,9 +24929,14 @@
           <t>tbd</t>
         </is>
       </c>
+      <c r="AC34" s="2" t="inlineStr">
+        <is>
+          <t>_3153</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB34"/>
+  <autoFilter ref="A1:AC34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23073,7 +24947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23086,6 +24960,7 @@
     <col width="29" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23139,6 +25014,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CDD Ref</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -23192,6 +25072,11 @@
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>_3028@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -23245,6 +25130,11 @@
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>_3032@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -23295,6 +25185,11 @@
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>_3036@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -23345,6 +25240,11 @@
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>_3040@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -23396,6 +25296,11 @@
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>_3044@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -23446,6 +25351,11 @@
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>_3048@_2995</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -23494,6 +25404,11 @@
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>_3112@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -23547,6 +25462,11 @@
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>_3114@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -23597,6 +25517,11 @@
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>_3118@_3053</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -23641,6 +25566,11 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>_3186@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -23685,6 +25615,11 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>_3188@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -23729,6 +25664,11 @@
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>_3190@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -23777,6 +25717,11 @@
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>_3192@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -23821,6 +25766,11 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>_3194@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -23865,6 +25815,11 @@
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>_3196@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -23909,6 +25864,11 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>_3198@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -23957,6 +25917,11 @@
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>_3200@_3159</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -24007,9 +25972,14 @@
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>_3202@_3159</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J19"/>
+  <autoFilter ref="A1:K19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>